<commit_message>
holdings_XLK.xlsx: EMEA UCITS Proxy (XLK) — 19.07.2026
</commit_message>
<xml_diff>
--- a/data/holdings_XLK.xlsx
+++ b/data/holdings_XLK.xlsx
@@ -35,7 +35,7 @@
     <t>Holdings As Of:</t>
   </si>
   <si>
-    <t>09-Jul-2026</t>
+    <t>16-Jul-2026</t>
   </si>
   <si>
     <t>ISIN</t>
@@ -152,6 +152,15 @@
     <t>Intel Corporation</t>
   </si>
   <si>
+    <t>US0382221051</t>
+  </si>
+  <si>
+    <t>2046552</t>
+  </si>
+  <si>
+    <t>Applied Materials Inc.</t>
+  </si>
+  <si>
     <t>US17275R1023</t>
   </si>
   <si>
@@ -164,15 +173,6 @@
     <t>Communications Equipment</t>
   </si>
   <si>
-    <t>US0382221051</t>
-  </si>
-  <si>
-    <t>2046552</t>
-  </si>
-  <si>
-    <t>Applied Materials Inc.</t>
-  </si>
-  <si>
     <t>US5128073062</t>
   </si>
   <si>
@@ -182,6 +182,24 @@
     <t>Lam Research Corporation</t>
   </si>
   <si>
+    <t>US69608A1088</t>
+  </si>
+  <si>
+    <t>BN78DQ4</t>
+  </si>
+  <si>
+    <t>Palantir Technologies Inc. Class A</t>
+  </si>
+  <si>
+    <t>US6974351057</t>
+  </si>
+  <si>
+    <t>B87ZMX0</t>
+  </si>
+  <si>
+    <t>Palo Alto Networks Inc.</t>
+  </si>
+  <si>
     <t>US4824801009</t>
   </si>
   <si>
@@ -191,15 +209,6 @@
     <t>KLA Corporation</t>
   </si>
   <si>
-    <t>US69608A1088</t>
-  </si>
-  <si>
-    <t>BN78DQ4</t>
-  </si>
-  <si>
-    <t>Palantir Technologies Inc. Class A</t>
-  </si>
-  <si>
     <t>US8825081040</t>
   </si>
   <si>
@@ -209,6 +218,33 @@
     <t>Texas Instruments Incorporated</t>
   </si>
   <si>
+    <t>US68389X1054</t>
+  </si>
+  <si>
+    <t>2661568</t>
+  </si>
+  <si>
+    <t>Oracle Corporation</t>
+  </si>
+  <si>
+    <t>US80004C2008</t>
+  </si>
+  <si>
+    <t>BSNPZV3</t>
+  </si>
+  <si>
+    <t>Sandisk Corporation</t>
+  </si>
+  <si>
+    <t>US22788C1053</t>
+  </si>
+  <si>
+    <t>BJJP138</t>
+  </si>
+  <si>
+    <t>CrowdStrike Holdings Inc. Class A</t>
+  </si>
+  <si>
     <t>US4592001014</t>
   </si>
   <si>
@@ -221,31 +257,52 @@
     <t>It Services</t>
   </si>
   <si>
-    <t>US80004C2008</t>
-  </si>
-  <si>
-    <t>BSNPZV3</t>
-  </si>
-  <si>
-    <t>Sandisk Corporation</t>
-  </si>
-  <si>
-    <t>US6974351057</t>
-  </si>
-  <si>
-    <t>B87ZMX0</t>
-  </si>
-  <si>
-    <t>Palo Alto Networks Inc.</t>
-  </si>
-  <si>
-    <t>US68389X1054</t>
-  </si>
-  <si>
-    <t>2661568</t>
-  </si>
-  <si>
-    <t>Oracle Corporation</t>
+    <t>US0320951017</t>
+  </si>
+  <si>
+    <t>2145084</t>
+  </si>
+  <si>
+    <t>Amphenol Corporation Class A</t>
+  </si>
+  <si>
+    <t>Electronic Equipment Instruments &amp; Components</t>
+  </si>
+  <si>
+    <t>US0326541051</t>
+  </si>
+  <si>
+    <t>2032067</t>
+  </si>
+  <si>
+    <t>Analog Devices Inc.</t>
+  </si>
+  <si>
+    <t>US7475251036</t>
+  </si>
+  <si>
+    <t>2714923</t>
+  </si>
+  <si>
+    <t>QUALCOMM Incorporated</t>
+  </si>
+  <si>
+    <t>US0404132054</t>
+  </si>
+  <si>
+    <t>BL9XPM3</t>
+  </si>
+  <si>
+    <t>Arista Networks Inc</t>
+  </si>
+  <si>
+    <t>IE00BKVD2N49</t>
+  </si>
+  <si>
+    <t>BKVD2N4</t>
+  </si>
+  <si>
+    <t>Seagate Technology Holdings PLC</t>
   </si>
   <si>
     <t>US5738741041</t>
@@ -257,45 +314,6 @@
     <t>Marvell Technology Inc.</t>
   </si>
   <si>
-    <t>US22788C1053</t>
-  </si>
-  <si>
-    <t>BJJP138</t>
-  </si>
-  <si>
-    <t>CrowdStrike Holdings Inc. Class A</t>
-  </si>
-  <si>
-    <t>US7475251036</t>
-  </si>
-  <si>
-    <t>2714923</t>
-  </si>
-  <si>
-    <t>QUALCOMM Incorporated</t>
-  </si>
-  <si>
-    <t>US0320951017</t>
-  </si>
-  <si>
-    <t>2145084</t>
-  </si>
-  <si>
-    <t>Amphenol Corporation Class A</t>
-  </si>
-  <si>
-    <t>Electronic Equipment Instruments &amp; Components</t>
-  </si>
-  <si>
-    <t>IE00BKVD2N49</t>
-  </si>
-  <si>
-    <t>BKVD2N4</t>
-  </si>
-  <si>
-    <t>Seagate Technology Holdings PLC</t>
-  </si>
-  <si>
     <t>US9581021055</t>
   </si>
   <si>
@@ -305,22 +323,13 @@
     <t>Western Digital Corporation</t>
   </si>
   <si>
-    <t>US0326541051</t>
-  </si>
-  <si>
-    <t>2032067</t>
-  </si>
-  <si>
-    <t>Analog Devices Inc.</t>
-  </si>
-  <si>
-    <t>US0404132054</t>
-  </si>
-  <si>
-    <t>BL9XPM3</t>
-  </si>
-  <si>
-    <t>Arista Networks Inc</t>
+    <t>US79466L3024</t>
+  </si>
+  <si>
+    <t>2310525</t>
+  </si>
+  <si>
+    <t>Salesforce Inc.</t>
   </si>
   <si>
     <t>US2193501051</t>
@@ -341,15 +350,6 @@
     <t>AppLovin Corp. Class A</t>
   </si>
   <si>
-    <t>US79466L3024</t>
-  </si>
-  <si>
-    <t>2310525</t>
-  </si>
-  <si>
-    <t>Salesforce Inc.</t>
-  </si>
-  <si>
     <t>US24703L2025</t>
   </si>
   <si>
@@ -395,6 +395,15 @@
     <t>Adobe Inc.</t>
   </si>
   <si>
+    <t>IE00B4BNMY34</t>
+  </si>
+  <si>
+    <t>B4BNMY3</t>
+  </si>
+  <si>
+    <t>Accenture Plc Class A</t>
+  </si>
+  <si>
     <t>US23804L1035</t>
   </si>
   <si>
@@ -404,13 +413,13 @@
     <t>Datadog Inc. Class A</t>
   </si>
   <si>
-    <t>IE00B4BNMY34</t>
-  </si>
-  <si>
-    <t>B4BNMY3</t>
-  </si>
-  <si>
-    <t>Accenture Plc Class A</t>
+    <t>US4612021034</t>
+  </si>
+  <si>
+    <t>2459020</t>
+  </si>
+  <si>
+    <t>Intuit Inc.</t>
   </si>
   <si>
     <t>US8716071076</t>
@@ -422,13 +431,13 @@
     <t>Synopsys Inc.</t>
   </si>
   <si>
-    <t>US4612021034</t>
-  </si>
-  <si>
-    <t>2459020</t>
-  </si>
-  <si>
-    <t>Intuit Inc.</t>
+    <t>US6200763075</t>
+  </si>
+  <si>
+    <t>B5BKPQ4</t>
+  </si>
+  <si>
+    <t>Motorola Solutions Inc.</t>
   </si>
   <si>
     <t>NL0009538784</t>
@@ -440,15 +449,6 @@
     <t>NXP Semiconductors NV</t>
   </si>
   <si>
-    <t>US6200763075</t>
-  </si>
-  <si>
-    <t>B5BKPQ4</t>
-  </si>
-  <si>
-    <t>Motorola Solutions Inc.</t>
-  </si>
-  <si>
     <t>US6098391054</t>
   </si>
   <si>
@@ -458,6 +458,24 @@
     <t>Monolithic Power Systems Inc.</t>
   </si>
   <si>
+    <t>US42824C1099</t>
+  </si>
+  <si>
+    <t>BYVYWS0</t>
+  </si>
+  <si>
+    <t>Hewlett Packard Enterprise Co.</t>
+  </si>
+  <si>
+    <t>IE000IVNQZ81</t>
+  </si>
+  <si>
+    <t>BRC3N84</t>
+  </si>
+  <si>
+    <t>TE Connectivity plc</t>
+  </si>
+  <si>
     <t>US1717793095</t>
   </si>
   <si>
@@ -467,13 +485,13 @@
     <t>Ciena Corporation</t>
   </si>
   <si>
-    <t>US42824C1099</t>
-  </si>
-  <si>
-    <t>BYVYWS0</t>
-  </si>
-  <si>
-    <t>Hewlett Packard Enterprise Co.</t>
+    <t>US55024U1097</t>
+  </si>
+  <si>
+    <t>BYM9ZP2</t>
+  </si>
+  <si>
+    <t>Lumentum Holdings Inc.</t>
   </si>
   <si>
     <t>US19247G1076</t>
@@ -485,22 +503,13 @@
     <t>Coherent Corp.</t>
   </si>
   <si>
-    <t>US55024U1097</t>
-  </si>
-  <si>
-    <t>BYM9ZP2</t>
-  </si>
-  <si>
-    <t>Lumentum Holdings Inc.</t>
-  </si>
-  <si>
-    <t>IE000IVNQZ81</t>
-  </si>
-  <si>
-    <t>BRC3N84</t>
-  </si>
-  <si>
-    <t>TE Connectivity plc</t>
+    <t>US49338L1035</t>
+  </si>
+  <si>
+    <t>BQZJ0Q9</t>
+  </si>
+  <si>
+    <t>Keysight Technologies Inc</t>
   </si>
   <si>
     <t>US8807701029</t>
@@ -512,13 +521,13 @@
     <t>Teradyne Inc.</t>
   </si>
   <si>
-    <t>US49338L1035</t>
-  </si>
-  <si>
-    <t>BQZJ0Q9</t>
-  </si>
-  <si>
-    <t>Keysight Technologies Inc</t>
+    <t>US0527691069</t>
+  </si>
+  <si>
+    <t>2065159</t>
+  </si>
+  <si>
+    <t>Autodesk Inc.</t>
   </si>
   <si>
     <t>SG9999000020</t>
@@ -539,13 +548,13 @@
     <t>Microchip Technology Incorporated</t>
   </si>
   <si>
-    <t>US0527691069</t>
-  </si>
-  <si>
-    <t>2065159</t>
-  </si>
-  <si>
-    <t>Autodesk Inc.</t>
+    <t>US7766961061</t>
+  </si>
+  <si>
+    <t>2749602</t>
+  </si>
+  <si>
+    <t>Roper Technologies Inc.</t>
   </si>
   <si>
     <t>US6821891057</t>
@@ -557,15 +566,6 @@
     <t>ON Semiconductor Corporation</t>
   </si>
   <si>
-    <t>US7766961061</t>
-  </si>
-  <si>
-    <t>2749602</t>
-  </si>
-  <si>
-    <t>Roper Technologies Inc.</t>
-  </si>
-  <si>
     <t>US4663131039</t>
   </si>
   <si>
@@ -584,6 +584,33 @@
     <t>NetApp Inc.</t>
   </si>
   <si>
+    <t>US98138H1014</t>
+  </si>
+  <si>
+    <t>B8K6ZD1</t>
+  </si>
+  <si>
+    <t>Workday Inc. Class A</t>
+  </si>
+  <si>
+    <t>US8793601050</t>
+  </si>
+  <si>
+    <t>2503477</t>
+  </si>
+  <si>
+    <t>Teledyne Technologies Incorporated</t>
+  </si>
+  <si>
+    <t>US3032501047</t>
+  </si>
+  <si>
+    <t>2330299</t>
+  </si>
+  <si>
+    <t>Fair Isaac Corporation</t>
+  </si>
+  <si>
     <t>US74743L1008</t>
   </si>
   <si>
@@ -593,33 +620,6 @@
     <t>Qnity Electronics Inc.</t>
   </si>
   <si>
-    <t>US3032501047</t>
-  </si>
-  <si>
-    <t>2330299</t>
-  </si>
-  <si>
-    <t>Fair Isaac Corporation</t>
-  </si>
-  <si>
-    <t>US8793601050</t>
-  </si>
-  <si>
-    <t>2503477</t>
-  </si>
-  <si>
-    <t>Teledyne Technologies Incorporated</t>
-  </si>
-  <si>
-    <t>US98138H1014</t>
-  </si>
-  <si>
-    <t>B8K6ZD1</t>
-  </si>
-  <si>
-    <t>Workday Inc. Class A</t>
-  </si>
-  <si>
     <t>US3364331070</t>
   </si>
   <si>
@@ -683,6 +683,24 @@
     <t>CDW Corporation</t>
   </si>
   <si>
+    <t>US6687711084</t>
+  </si>
+  <si>
+    <t>BJN4XN5</t>
+  </si>
+  <si>
+    <t>Gen Digital Inc.</t>
+  </si>
+  <si>
+    <t>US69370C1009</t>
+  </si>
+  <si>
+    <t>B95N910</t>
+  </si>
+  <si>
+    <t>PTC Inc.</t>
+  </si>
+  <si>
     <t>US86800U3023</t>
   </si>
   <si>
@@ -692,24 +710,6 @@
     <t>Super Micro Computer Inc.</t>
   </si>
   <si>
-    <t>US6687711084</t>
-  </si>
-  <si>
-    <t>BJN4XN5</t>
-  </si>
-  <si>
-    <t>Gen Digital Inc.</t>
-  </si>
-  <si>
-    <t>US69370C1009</t>
-  </si>
-  <si>
-    <t>B95N910</t>
-  </si>
-  <si>
-    <t>PTC Inc.</t>
-  </si>
-  <si>
     <t>US9022521051</t>
   </si>
   <si>
@@ -719,6 +719,15 @@
     <t>Tyler Technologies Inc.</t>
   </si>
   <si>
+    <t>US3802371076</t>
+  </si>
+  <si>
+    <t>BWFRFC6</t>
+  </si>
+  <si>
+    <t>GoDaddy Inc. Class A</t>
+  </si>
+  <si>
     <t>US9892071054</t>
   </si>
   <si>
@@ -737,13 +746,13 @@
     <t>Trimble Inc.</t>
   </si>
   <si>
-    <t>US3802371076</t>
-  </si>
-  <si>
-    <t>BWFRFC6</t>
-  </si>
-  <si>
-    <t>GoDaddy Inc. Class A</t>
+    <t>US3666511072</t>
+  </si>
+  <si>
+    <t>2372763</t>
+  </si>
+  <si>
+    <t>Gartner Inc.</t>
   </si>
   <si>
     <t>US83088M1027</t>
@@ -753,15 +762,6 @@
   </si>
   <si>
     <t>Skyworks Solutions Inc.</t>
-  </si>
-  <si>
-    <t>US3666511072</t>
-  </si>
-  <si>
-    <t>2372763</t>
-  </si>
-  <si>
-    <t>Gartner Inc.</t>
   </si>
   <si>
     <t>Unassigned</t>
@@ -2059,16 +2059,16 @@
         <v>22</v>
       </c>
       <c r="E7" t="n" s="2">
-        <v>2038979.0</v>
+        <v>2041695.0</v>
       </c>
       <c r="F7" t="n" s="3">
-        <v>20.148515</v>
+        <v>21.055765</v>
       </c>
       <c r="G7" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H7" t="n" s="4">
-        <v>202.78</v>
+        <v>207.4</v>
       </c>
       <c r="I7" t="s" s="1">
         <v>24</v>
@@ -2077,7 +2077,7 @@
         <v>25</v>
       </c>
       <c r="K7" t="n" s="5">
-        <v>4.1346416E8</v>
+        <v>4.2344755E8</v>
       </c>
     </row>
     <row r="8">
@@ -2094,16 +2094,16 @@
         <v>22</v>
       </c>
       <c r="E8" t="n" s="6">
-        <v>1236437.0</v>
+        <v>1238084.0</v>
       </c>
       <c r="F8" t="n" s="7">
-        <v>19.053137</v>
+        <v>20.516568</v>
       </c>
       <c r="G8" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H8" t="n" s="8">
-        <v>316.22</v>
+        <v>333.26</v>
       </c>
       <c r="I8" t="s" s="1">
         <v>24</v>
@@ -2112,7 +2112,7 @@
         <v>29</v>
       </c>
       <c r="K8" t="n" s="9">
-        <v>3.909861E8</v>
+        <v>4.1260387E8</v>
       </c>
     </row>
     <row r="9">
@@ -2129,16 +2129,16 @@
         <v>22</v>
       </c>
       <c r="E9" t="n" s="10">
-        <v>625354.0</v>
+        <v>626187.0</v>
       </c>
       <c r="F9" t="n" s="11">
-        <v>11.713031</v>
+        <v>12.489013</v>
       </c>
       <c r="G9" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H9" t="n" s="12">
-        <v>384.36</v>
+        <v>401.1</v>
       </c>
       <c r="I9" t="s" s="1">
         <v>24</v>
@@ -2147,7 +2147,7 @@
         <v>33</v>
       </c>
       <c r="K9" t="n" s="13">
-        <v>2.4036106E8</v>
+        <v>2.511636E8</v>
       </c>
     </row>
     <row r="10">
@@ -2164,16 +2164,16 @@
         <v>22</v>
       </c>
       <c r="E10" t="n" s="14">
-        <v>398583.0</v>
+        <v>399114.0</v>
       </c>
       <c r="F10" t="n" s="15">
-        <v>7.790896</v>
+        <v>7.431256</v>
       </c>
       <c r="G10" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H10" t="n" s="16">
-        <v>401.11</v>
+        <v>374.45</v>
       </c>
       <c r="I10" t="s" s="1">
         <v>24</v>
@@ -2182,7 +2182,7 @@
         <v>25</v>
       </c>
       <c r="K10" t="n" s="17">
-        <v>1.5987563E8</v>
+        <v>1.4944824E8</v>
       </c>
     </row>
     <row r="11">
@@ -2199,16 +2199,16 @@
         <v>22</v>
       </c>
       <c r="E11" t="n" s="18">
-        <v>94930.0</v>
+        <v>95056.0</v>
       </c>
       <c r="F11" t="n" s="19">
-        <v>4.587359</v>
+        <v>4.032755</v>
       </c>
       <c r="G11" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H11" t="n" s="20">
-        <v>991.64</v>
+        <v>853.2</v>
       </c>
       <c r="I11" t="s" s="1">
         <v>24</v>
@@ -2217,7 +2217,7 @@
         <v>25</v>
       </c>
       <c r="K11" t="n" s="21">
-        <v>9.413638E7</v>
+        <v>8.110178E7</v>
       </c>
     </row>
     <row r="12">
@@ -2234,16 +2234,16 @@
         <v>22</v>
       </c>
       <c r="E12" t="n" s="22">
-        <v>137272.0</v>
+        <v>137455.0</v>
       </c>
       <c r="F12" t="n" s="23">
-        <v>3.657228</v>
+        <v>3.423873</v>
       </c>
       <c r="G12" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H12" t="n" s="24">
-        <v>546.72</v>
+        <v>500.94</v>
       </c>
       <c r="I12" t="s" s="1">
         <v>24</v>
@@ -2252,7 +2252,7 @@
         <v>25</v>
       </c>
       <c r="K12" t="n" s="25">
-        <v>7.504934E7</v>
+        <v>6.88567E7</v>
       </c>
     </row>
     <row r="13">
@@ -2269,16 +2269,16 @@
         <v>22</v>
       </c>
       <c r="E13" t="n" s="26">
-        <v>397724.0</v>
+        <v>398254.0</v>
       </c>
       <c r="F13" t="n" s="27">
-        <v>2.181192</v>
+        <v>1.920497</v>
       </c>
       <c r="G13" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H13" t="n" s="28">
-        <v>112.54</v>
+        <v>96.98</v>
       </c>
       <c r="I13" t="s" s="1">
         <v>24</v>
@@ -2287,7 +2287,7 @@
         <v>25</v>
       </c>
       <c r="K13" t="n" s="29">
-        <v>4.475986E7</v>
+        <v>3.862267E7</v>
       </c>
     </row>
     <row r="14">
@@ -2304,60 +2304,60 @@
         <v>22</v>
       </c>
       <c r="E14" t="n" s="30">
-        <v>332518.0</v>
+        <v>66898.0</v>
       </c>
       <c r="F14" t="n" s="31">
-        <v>1.917087</v>
+        <v>1.865921</v>
       </c>
       <c r="G14" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H14" t="n" s="32">
-        <v>118.31</v>
+        <v>560.93</v>
       </c>
       <c r="I14" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J14" t="s" s="1">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n" s="33">
-        <v>3.9340204E7</v>
+        <v>3.7525096E7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="1">
+        <v>49</v>
+      </c>
+      <c r="B15" t="s" s="1">
         <v>50</v>
       </c>
-      <c r="B15" t="s" s="1">
+      <c r="C15" t="s" s="1">
         <v>51</v>
       </c>
-      <c r="C15" t="s" s="1">
+      <c r="D15" t="s" s="1">
+        <v>22</v>
+      </c>
+      <c r="E15" t="n" s="34">
+        <v>332961.0</v>
+      </c>
+      <c r="F15" t="n" s="35">
+        <v>1.81557</v>
+      </c>
+      <c r="G15" t="s" s="1">
+        <v>23</v>
+      </c>
+      <c r="H15" t="n" s="36">
+        <v>109.66</v>
+      </c>
+      <c r="I15" t="s" s="1">
+        <v>24</v>
+      </c>
+      <c r="J15" t="s" s="1">
         <v>52</v>
       </c>
-      <c r="D15" t="s" s="1">
-        <v>22</v>
-      </c>
-      <c r="E15" t="n" s="34">
-        <v>66809.0</v>
-      </c>
-      <c r="F15" t="n" s="35">
-        <v>1.916482</v>
-      </c>
-      <c r="G15" t="s" s="1">
-        <v>23</v>
-      </c>
-      <c r="H15" t="n" s="36">
-        <v>588.66</v>
-      </c>
-      <c r="I15" t="s" s="1">
-        <v>24</v>
-      </c>
-      <c r="J15" t="s" s="1">
-        <v>25</v>
-      </c>
       <c r="K15" t="n" s="37">
-        <v>3.9327784E7</v>
+        <v>3.6512504E7</v>
       </c>
     </row>
     <row r="16">
@@ -2374,16 +2374,16 @@
         <v>22</v>
       </c>
       <c r="E16" t="n" s="38">
-        <v>105275.0</v>
+        <v>105415.0</v>
       </c>
       <c r="F16" t="n" s="39">
-        <v>1.811817</v>
+        <v>1.682382</v>
       </c>
       <c r="G16" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H16" t="n" s="40">
-        <v>353.17</v>
+        <v>320.96</v>
       </c>
       <c r="I16" t="s" s="1">
         <v>24</v>
@@ -2392,7 +2392,7 @@
         <v>25</v>
       </c>
       <c r="K16" t="n" s="41">
-        <v>3.7179972E7</v>
+        <v>3.3834E7</v>
       </c>
     </row>
     <row r="17">
@@ -2409,25 +2409,25 @@
         <v>22</v>
       </c>
       <c r="E17" t="n" s="42">
-        <v>109965.0</v>
+        <v>193546.0</v>
       </c>
       <c r="F17" t="n" s="43">
-        <v>1.229929</v>
+        <v>1.293851</v>
       </c>
       <c r="G17" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H17" t="n" s="44">
-        <v>229.52</v>
+        <v>134.44</v>
       </c>
       <c r="I17" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J17" t="s" s="1">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="K17" t="n" s="45">
-        <v>2.5239166E7</v>
+        <v>2.6020324E7</v>
       </c>
     </row>
     <row r="18">
@@ -2444,16 +2444,16 @@
         <v>22</v>
       </c>
       <c r="E18" t="n" s="46">
-        <v>193289.0</v>
+        <v>68365.0</v>
       </c>
       <c r="F18" t="n" s="47">
-        <v>1.215449</v>
+        <v>1.203362</v>
       </c>
       <c r="G18" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H18" t="n" s="48">
-        <v>129.04</v>
+        <v>353.99</v>
       </c>
       <c r="I18" t="s" s="1">
         <v>24</v>
@@ -2462,7 +2462,7 @@
         <v>33</v>
       </c>
       <c r="K18" t="n" s="49">
-        <v>2.4942012E7</v>
+        <v>2.4200526E7</v>
       </c>
     </row>
     <row r="19">
@@ -2479,16 +2479,16 @@
         <v>22</v>
       </c>
       <c r="E19" t="n" s="50">
-        <v>76614.0</v>
+        <v>110111.0</v>
       </c>
       <c r="F19" t="n" s="51">
-        <v>1.151889</v>
+        <v>1.201101</v>
       </c>
       <c r="G19" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H19" t="n" s="52">
-        <v>308.53</v>
+        <v>219.37</v>
       </c>
       <c r="I19" t="s" s="1">
         <v>24</v>
@@ -2497,7 +2497,7 @@
         <v>25</v>
       </c>
       <c r="K19" t="n" s="53">
-        <v>2.3637718E7</v>
+        <v>2.415505E7</v>
       </c>
     </row>
     <row r="20">
@@ -2514,121 +2514,121 @@
         <v>22</v>
       </c>
       <c r="E20" t="n" s="54">
-        <v>79118.0</v>
+        <v>76716.0</v>
       </c>
       <c r="F20" t="n" s="55">
-        <v>1.138529</v>
+        <v>1.110909</v>
       </c>
       <c r="G20" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H20" t="n" s="56">
-        <v>295.3</v>
+        <v>291.22</v>
       </c>
       <c r="I20" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J20" t="s" s="1">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="K20" t="n" s="57">
-        <v>2.3363546E7</v>
+        <v>2.2341234E7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="1">
+        <v>68</v>
+      </c>
+      <c r="B21" t="s" s="1">
         <v>69</v>
       </c>
-      <c r="B21" t="s" s="1">
+      <c r="C21" t="s" s="1">
         <v>70</v>
       </c>
-      <c r="C21" t="s" s="1">
-        <v>71</v>
-      </c>
       <c r="D21" t="s" s="1">
         <v>22</v>
       </c>
       <c r="E21" t="n" s="58">
-        <v>12472.0</v>
+        <v>143035.0</v>
       </c>
       <c r="F21" t="n" s="59">
-        <v>1.129406</v>
+        <v>0.883426</v>
       </c>
       <c r="G21" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H21" t="n" s="60">
-        <v>1858.27</v>
+        <v>124.21</v>
       </c>
       <c r="I21" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J21" t="s" s="1">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K21" t="n" s="61">
-        <v>2.3176344E7</v>
+        <v>1.7766378E7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="1">
+        <v>71</v>
+      </c>
+      <c r="B22" t="s" s="1">
         <v>72</v>
       </c>
-      <c r="B22" t="s" s="1">
+      <c r="C22" t="s" s="1">
         <v>73</v>
       </c>
-      <c r="C22" t="s" s="1">
-        <v>74</v>
-      </c>
       <c r="D22" t="s" s="1">
         <v>22</v>
       </c>
       <c r="E22" t="n" s="62">
-        <v>68274.0</v>
+        <v>12489.0</v>
       </c>
       <c r="F22" t="n" s="63">
-        <v>1.125577</v>
+        <v>0.876296</v>
       </c>
       <c r="G22" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H22" t="n" s="64">
-        <v>338.31</v>
+        <v>1411.08</v>
       </c>
       <c r="I22" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J22" t="s" s="1">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="K22" t="n" s="65">
-        <v>2.3097776E7</v>
+        <v>1.7622978E7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="1">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s" s="1">
         <v>75</v>
       </c>
-      <c r="B23" t="s" s="1">
+      <c r="C23" t="s" s="1">
         <v>76</v>
       </c>
-      <c r="C23" t="s" s="1">
-        <v>77</v>
-      </c>
       <c r="D23" t="s" s="1">
         <v>22</v>
       </c>
       <c r="E23" t="n" s="66">
-        <v>142845.0</v>
+        <v>85844.0</v>
       </c>
       <c r="F23" t="n" s="67">
-        <v>1.003912</v>
+        <v>0.869762</v>
       </c>
       <c r="G23" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H23" t="n" s="68">
-        <v>144.22</v>
+        <v>203.76</v>
       </c>
       <c r="I23" t="s" s="1">
         <v>24</v>
@@ -2637,42 +2637,42 @@
         <v>33</v>
       </c>
       <c r="K23" t="n" s="69">
-        <v>2.0601106E7</v>
+        <v>1.7491574E7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="1">
+        <v>77</v>
+      </c>
+      <c r="B24" t="s" s="1">
         <v>78</v>
       </c>
-      <c r="B24" t="s" s="1">
+      <c r="C24" t="s" s="1">
         <v>79</v>
       </c>
-      <c r="C24" t="s" s="1">
+      <c r="D24" t="s" s="1">
+        <v>22</v>
+      </c>
+      <c r="E24" t="n" s="70">
+        <v>79223.0</v>
+      </c>
+      <c r="F24" t="n" s="71">
+        <v>0.862911</v>
+      </c>
+      <c r="G24" t="s" s="1">
+        <v>23</v>
+      </c>
+      <c r="H24" t="n" s="72">
+        <v>219.05</v>
+      </c>
+      <c r="I24" t="s" s="1">
+        <v>24</v>
+      </c>
+      <c r="J24" t="s" s="1">
         <v>80</v>
       </c>
-      <c r="D24" t="s" s="1">
-        <v>22</v>
-      </c>
-      <c r="E24" t="n" s="70">
-        <v>73705.0</v>
-      </c>
-      <c r="F24" t="n" s="71">
-        <v>0.873757</v>
-      </c>
-      <c r="G24" t="s" s="1">
-        <v>23</v>
-      </c>
-      <c r="H24" t="n" s="72">
-        <v>243.27</v>
-      </c>
-      <c r="I24" t="s" s="1">
-        <v>24</v>
-      </c>
-      <c r="J24" t="s" s="1">
-        <v>25</v>
-      </c>
       <c r="K24" t="n" s="73">
-        <v>1.7930216E7</v>
+        <v>1.7353798E7</v>
       </c>
     </row>
     <row r="25">
@@ -2689,51 +2689,51 @@
         <v>22</v>
       </c>
       <c r="E25" t="n" s="74">
-        <v>85730.0</v>
+        <v>103704.0</v>
       </c>
       <c r="F25" t="n" s="75">
-        <v>0.828857</v>
+        <v>0.789688</v>
       </c>
       <c r="G25" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H25" t="n" s="76">
-        <v>198.4</v>
+        <v>153.14</v>
       </c>
       <c r="I25" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J25" t="s" s="1">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="K25" t="n" s="77">
-        <v>1.7008832E7</v>
+        <v>1.5881231E7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="1">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s" s="1">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s" s="1">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D26" t="s" s="1">
         <v>22</v>
       </c>
       <c r="E26" t="n" s="78">
-        <v>88727.0</v>
+        <v>41157.0</v>
       </c>
       <c r="F26" t="n" s="79">
-        <v>0.826313</v>
+        <v>0.778761</v>
       </c>
       <c r="G26" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H26" t="n" s="80">
-        <v>191.11</v>
+        <v>380.53</v>
       </c>
       <c r="I26" t="s" s="1">
         <v>24</v>
@@ -2742,42 +2742,42 @@
         <v>25</v>
       </c>
       <c r="K26" t="n" s="81">
-        <v>1.6956616E7</v>
+        <v>1.5661473E7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="1">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B27" t="s" s="1">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s" s="1">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s" s="1">
         <v>22</v>
       </c>
       <c r="E27" t="n" s="82">
-        <v>103566.0</v>
+        <v>88845.0</v>
       </c>
       <c r="F27" t="n" s="83">
-        <v>0.818805</v>
+        <v>0.753718</v>
       </c>
       <c r="G27" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H27" t="n" s="84">
-        <v>162.24</v>
+        <v>170.61</v>
       </c>
       <c r="I27" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J27" t="s" s="1">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="K27" t="n" s="85">
-        <v>1.6802548E7</v>
+        <v>1.5157845E7</v>
       </c>
     </row>
     <row r="28">
@@ -2794,25 +2794,25 @@
         <v>22</v>
       </c>
       <c r="E28" t="n" s="86">
-        <v>18874.0</v>
+        <v>87043.0</v>
       </c>
       <c r="F28" t="n" s="87">
-        <v>0.818659</v>
+        <v>0.729558</v>
       </c>
       <c r="G28" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H28" t="n" s="88">
-        <v>890.09</v>
+        <v>168.56</v>
       </c>
       <c r="I28" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J28" t="s" s="1">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="K28" t="n" s="89">
-        <v>1.6799558E7</v>
+        <v>1.4671968E7</v>
       </c>
     </row>
     <row r="29">
@@ -2829,16 +2829,16 @@
         <v>22</v>
       </c>
       <c r="E29" t="n" s="90">
-        <v>29022.0</v>
+        <v>18899.0</v>
       </c>
       <c r="F29" t="n" s="91">
-        <v>0.817519</v>
+        <v>0.700571</v>
       </c>
       <c r="G29" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H29" t="n" s="92">
-        <v>578.05</v>
+        <v>745.49</v>
       </c>
       <c r="I29" t="s" s="1">
         <v>24</v>
@@ -2847,7 +2847,7 @@
         <v>29</v>
       </c>
       <c r="K29" t="n" s="93">
-        <v>1.6776167E7</v>
+        <v>1.4089016E7</v>
       </c>
     </row>
     <row r="30">
@@ -2864,16 +2864,16 @@
         <v>22</v>
       </c>
       <c r="E30" t="n" s="94">
-        <v>41102.0</v>
+        <v>73803.0</v>
       </c>
       <c r="F30" t="n" s="95">
-        <v>0.788438</v>
+        <v>0.691028</v>
       </c>
       <c r="G30" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H30" t="n" s="96">
-        <v>393.64</v>
+        <v>188.3</v>
       </c>
       <c r="I30" t="s" s="1">
         <v>24</v>
@@ -2882,7 +2882,7 @@
         <v>25</v>
       </c>
       <c r="K30" t="n" s="97">
-        <v>1.6179391E7</v>
+        <v>1.3897105E7</v>
       </c>
     </row>
     <row r="31">
@@ -2899,25 +2899,25 @@
         <v>22</v>
       </c>
       <c r="E31" t="n" s="98">
-        <v>86927.0</v>
+        <v>29061.0</v>
       </c>
       <c r="F31" t="n" s="99">
-        <v>0.782354</v>
+        <v>0.674562</v>
       </c>
       <c r="G31" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H31" t="n" s="100">
-        <v>184.69</v>
+        <v>466.81</v>
       </c>
       <c r="I31" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J31" t="s" s="1">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="K31" t="n" s="101">
-        <v>1.6054548E7</v>
+        <v>1.3565965E7</v>
       </c>
     </row>
     <row r="32">
@@ -2934,25 +2934,25 @@
         <v>22</v>
       </c>
       <c r="E32" t="n" s="102">
-        <v>65934.0</v>
+        <v>68963.0</v>
       </c>
       <c r="F32" t="n" s="103">
-        <v>0.618122</v>
+        <v>0.592147</v>
       </c>
       <c r="G32" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H32" t="n" s="104">
-        <v>192.38</v>
+        <v>172.68</v>
       </c>
       <c r="I32" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J32" t="s" s="1">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="K32" t="n" s="105">
-        <v>1.2684383E7</v>
+        <v>1.1908531E7</v>
       </c>
     </row>
     <row r="33">
@@ -2969,25 +2969,25 @@
         <v>22</v>
       </c>
       <c r="E33" t="n" s="106">
-        <v>22647.0</v>
+        <v>66022.0</v>
       </c>
       <c r="F33" t="n" s="107">
-        <v>0.574352</v>
+        <v>0.519981</v>
       </c>
       <c r="G33" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H33" t="n" s="108">
-        <v>520.43</v>
+        <v>158.39</v>
       </c>
       <c r="I33" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J33" t="s" s="1">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="K33" t="n" s="109">
-        <v>1.1786178E7</v>
+        <v>1.0457225E7</v>
       </c>
     </row>
     <row r="34">
@@ -3004,16 +3004,16 @@
         <v>22</v>
       </c>
       <c r="E34" t="n" s="110">
-        <v>68871.0</v>
+        <v>22677.0</v>
       </c>
       <c r="F34" t="n" s="111">
-        <v>0.545375</v>
+        <v>0.489922</v>
       </c>
       <c r="G34" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H34" t="n" s="112">
-        <v>162.5</v>
+        <v>434.48</v>
       </c>
       <c r="I34" t="s" s="1">
         <v>24</v>
@@ -3022,7 +3022,7 @@
         <v>33</v>
       </c>
       <c r="K34" t="n" s="113">
-        <v>1.1191538E7</v>
+        <v>9852703.0</v>
       </c>
     </row>
     <row r="35">
@@ -3039,16 +3039,16 @@
         <v>22</v>
       </c>
       <c r="E35" t="n" s="114">
-        <v>24347.0</v>
+        <v>24379.0</v>
       </c>
       <c r="F35" t="n" s="115">
-        <v>0.534165</v>
+        <v>0.474445</v>
       </c>
       <c r="G35" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H35" t="n" s="116">
-        <v>450.22</v>
+        <v>391.38</v>
       </c>
       <c r="I35" t="s" s="1">
         <v>24</v>
@@ -3057,7 +3057,7 @@
         <v>29</v>
       </c>
       <c r="K35" t="n" s="117">
-        <v>1.0961506E7</v>
+        <v>9541453.0</v>
       </c>
     </row>
     <row r="36">
@@ -3074,16 +3074,16 @@
         <v>22</v>
       </c>
       <c r="E36" t="n" s="118">
-        <v>86824.0</v>
+        <v>86940.0</v>
       </c>
       <c r="F36" t="n" s="119">
-        <v>0.460504</v>
+        <v>0.449641</v>
       </c>
       <c r="G36" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H36" t="n" s="120">
-        <v>108.84</v>
+        <v>104.01</v>
       </c>
       <c r="I36" t="s" s="1">
         <v>24</v>
@@ -3092,7 +3092,7 @@
         <v>33</v>
       </c>
       <c r="K36" t="n" s="121">
-        <v>9449924.0</v>
+        <v>9042629.0</v>
       </c>
     </row>
     <row r="37">
@@ -3109,16 +3109,16 @@
         <v>22</v>
       </c>
       <c r="E37" t="n" s="122">
-        <v>23220.0</v>
+        <v>23251.0</v>
       </c>
       <c r="F37" t="n" s="123">
-        <v>0.436715</v>
+        <v>0.421589</v>
       </c>
       <c r="G37" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H37" t="n" s="124">
-        <v>385.95</v>
+        <v>364.65</v>
       </c>
       <c r="I37" t="s" s="1">
         <v>24</v>
@@ -3127,7 +3127,7 @@
         <v>33</v>
       </c>
       <c r="K37" t="n" s="125">
-        <v>8961759.0</v>
+        <v>8478477.0</v>
       </c>
     </row>
     <row r="38">
@@ -3144,16 +3144,16 @@
         <v>22</v>
       </c>
       <c r="E38" t="n" s="126">
-        <v>52428.0</v>
+        <v>52498.0</v>
       </c>
       <c r="F38" t="n" s="127">
-        <v>0.418309</v>
+        <v>0.419707</v>
       </c>
       <c r="G38" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H38" t="n" s="128">
-        <v>163.73</v>
+        <v>160.78</v>
       </c>
       <c r="I38" t="s" s="1">
         <v>24</v>
@@ -3162,7 +3162,7 @@
         <v>33</v>
       </c>
       <c r="K38" t="n" s="129">
-        <v>8584036.0</v>
+        <v>8440628.0</v>
       </c>
     </row>
     <row r="39">
@@ -3179,16 +3179,16 @@
         <v>22</v>
       </c>
       <c r="E39" t="n" s="130">
-        <v>34023.0</v>
+        <v>34068.0</v>
       </c>
       <c r="F39" t="n" s="131">
-        <v>0.369148</v>
+        <v>0.398619</v>
       </c>
       <c r="G39" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H39" t="n" s="132">
-        <v>222.65</v>
+        <v>235.31</v>
       </c>
       <c r="I39" t="s" s="1">
         <v>24</v>
@@ -3197,7 +3197,7 @@
         <v>33</v>
       </c>
       <c r="K39" t="n" s="133">
-        <v>7575221.0</v>
+        <v>8016541.0</v>
       </c>
     </row>
     <row r="40">
@@ -3214,25 +3214,25 @@
         <v>22</v>
       </c>
       <c r="E40" t="n" s="134">
-        <v>27849.0</v>
+        <v>51755.0</v>
       </c>
       <c r="F40" t="n" s="135">
-        <v>0.365062</v>
+        <v>0.372153</v>
       </c>
       <c r="G40" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H40" t="n" s="136">
-        <v>269.0</v>
+        <v>144.61</v>
       </c>
       <c r="I40" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J40" t="s" s="1">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="K40" t="n" s="137">
-        <v>7491381.0</v>
+        <v>7484290.5</v>
       </c>
     </row>
     <row r="41">
@@ -3249,25 +3249,25 @@
         <v>22</v>
       </c>
       <c r="E41" t="n" s="138">
-        <v>51686.0</v>
+        <v>27886.0</v>
       </c>
       <c r="F41" t="n" s="139">
-        <v>0.350252</v>
+        <v>0.363738</v>
       </c>
       <c r="G41" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H41" t="n" s="140">
-        <v>139.06</v>
+        <v>262.32</v>
       </c>
       <c r="I41" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J41" t="s" s="1">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="K41" t="n" s="141">
-        <v>7187455.0</v>
+        <v>7315055.5</v>
       </c>
     </row>
     <row r="42">
@@ -3284,16 +3284,16 @@
         <v>22</v>
       </c>
       <c r="E42" t="n" s="142">
-        <v>16120.0</v>
+        <v>23312.0</v>
       </c>
       <c r="F42" t="n" s="143">
-        <v>0.348286</v>
+        <v>0.341715</v>
       </c>
       <c r="G42" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H42" t="n" s="144">
-        <v>443.37</v>
+        <v>294.79</v>
       </c>
       <c r="I42" t="s" s="1">
         <v>24</v>
@@ -3302,7 +3302,7 @@
         <v>33</v>
       </c>
       <c r="K42" t="n" s="145">
-        <v>7147124.5</v>
+        <v>6872144.5</v>
       </c>
     </row>
     <row r="43">
@@ -3319,16 +3319,16 @@
         <v>22</v>
       </c>
       <c r="E43" t="n" s="146">
-        <v>23281.0</v>
+        <v>16141.0</v>
       </c>
       <c r="F43" t="n" s="147">
-        <v>0.310151</v>
+        <v>0.33471</v>
       </c>
       <c r="G43" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H43" t="n" s="148">
-        <v>273.38</v>
+        <v>417.03</v>
       </c>
       <c r="I43" t="s" s="1">
         <v>24</v>
@@ -3337,7 +3337,7 @@
         <v>33</v>
       </c>
       <c r="K43" t="n" s="149">
-        <v>6364560.0</v>
+        <v>6731281.0</v>
       </c>
     </row>
     <row r="44">
@@ -3354,25 +3354,25 @@
         <v>22</v>
       </c>
       <c r="E44" t="n" s="150">
-        <v>21250.0</v>
+        <v>13999.0</v>
       </c>
       <c r="F44" t="n" s="151">
-        <v>0.300864</v>
+        <v>0.288316</v>
       </c>
       <c r="G44" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H44" t="n" s="152">
-        <v>290.54</v>
+        <v>414.19</v>
       </c>
       <c r="I44" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J44" t="s" s="1">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="K44" t="n" s="153">
-        <v>6173975.0</v>
+        <v>5798246.0</v>
       </c>
     </row>
     <row r="45">
@@ -3389,25 +3389,25 @@
         <v>22</v>
       </c>
       <c r="E45" t="n" s="154">
-        <v>13980.0</v>
+        <v>21278.0</v>
       </c>
       <c r="F45" t="n" s="155">
-        <v>0.284228</v>
+        <v>0.286369</v>
       </c>
       <c r="G45" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H45" t="n" s="156">
-        <v>417.21</v>
+        <v>270.66</v>
       </c>
       <c r="I45" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J45" t="s" s="1">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="K45" t="n" s="157">
-        <v>5832596.0</v>
+        <v>5759103.5</v>
       </c>
     </row>
     <row r="46">
@@ -3424,16 +3424,16 @@
         <v>22</v>
       </c>
       <c r="E46" t="n" s="158">
-        <v>4143.0</v>
+        <v>4149.0</v>
       </c>
       <c r="F46" t="n" s="159">
-        <v>0.277426</v>
+        <v>0.269365</v>
       </c>
       <c r="G46" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H46" t="n" s="160">
-        <v>1374.13</v>
+        <v>1305.65</v>
       </c>
       <c r="I46" t="s" s="1">
         <v>24</v>
@@ -3442,7 +3442,7 @@
         <v>25</v>
       </c>
       <c r="K46" t="n" s="161">
-        <v>5693020.5</v>
+        <v>5417142.0</v>
       </c>
     </row>
     <row r="47">
@@ -3459,25 +3459,25 @@
         <v>22</v>
       </c>
       <c r="E47" t="n" s="162">
-        <v>11905.0</v>
+        <v>111852.0</v>
       </c>
       <c r="F47" t="n" s="163">
-        <v>0.268223</v>
+        <v>0.251004</v>
       </c>
       <c r="G47" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H47" t="n" s="164">
-        <v>462.34</v>
+        <v>45.13</v>
       </c>
       <c r="I47" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J47" t="s" s="1">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="K47" t="n" s="165">
-        <v>5504157.5</v>
+        <v>5047881.0</v>
       </c>
     </row>
     <row r="48">
@@ -3494,25 +3494,25 @@
         <v>22</v>
       </c>
       <c r="E48" t="n" s="166">
-        <v>111703.0</v>
+        <v>24610.0</v>
       </c>
       <c r="F48" t="n" s="167">
-        <v>0.267325</v>
+        <v>0.24789</v>
       </c>
       <c r="G48" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H48" t="n" s="168">
-        <v>49.11</v>
+        <v>202.57</v>
       </c>
       <c r="I48" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J48" t="s" s="1">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="K48" t="n" s="169">
-        <v>5485734.5</v>
+        <v>4985247.5</v>
       </c>
     </row>
     <row r="49">
@@ -3529,25 +3529,25 @@
         <v>22</v>
       </c>
       <c r="E49" t="n" s="170">
-        <v>16470.0</v>
+        <v>11921.0</v>
       </c>
       <c r="F49" t="n" s="171">
-        <v>0.262643</v>
+        <v>0.230474</v>
       </c>
       <c r="G49" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H49" t="n" s="172">
-        <v>327.24</v>
+        <v>388.81</v>
       </c>
       <c r="I49" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J49" t="s" s="1">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="K49" t="n" s="173">
-        <v>5389643.0</v>
+        <v>4635004.0</v>
       </c>
     </row>
     <row r="50">
@@ -3564,25 +3564,25 @@
         <v>22</v>
       </c>
       <c r="E50" t="n" s="174">
-        <v>6553.0</v>
+        <v>6562.0</v>
       </c>
       <c r="F50" t="n" s="175">
-        <v>0.250923</v>
+        <v>0.230438</v>
       </c>
       <c r="G50" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H50" t="n" s="176">
-        <v>785.77</v>
+        <v>706.23</v>
       </c>
       <c r="I50" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J50" t="s" s="1">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K50" t="n" s="177">
-        <v>5149151.0</v>
+        <v>4634281.5</v>
       </c>
     </row>
     <row r="51">
@@ -3599,25 +3599,25 @@
         <v>22</v>
       </c>
       <c r="E51" t="n" s="178">
-        <v>24577.0</v>
+        <v>16492.0</v>
       </c>
       <c r="F51" t="n" s="179">
-        <v>0.238227</v>
+        <v>0.227123</v>
       </c>
       <c r="G51" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H51" t="n" s="180">
-        <v>198.91</v>
+        <v>276.96</v>
       </c>
       <c r="I51" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J51" t="s" s="1">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="K51" t="n" s="181">
-        <v>4888611.0</v>
+        <v>4567624.5</v>
       </c>
     </row>
     <row r="52">
@@ -3634,25 +3634,25 @@
         <v>22</v>
       </c>
       <c r="E52" t="n" s="182">
-        <v>13185.0</v>
+        <v>14453.0</v>
       </c>
       <c r="F52" t="n" s="183">
-        <v>0.233073</v>
+        <v>0.224771</v>
       </c>
       <c r="G52" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H52" t="n" s="184">
-        <v>362.75</v>
+        <v>312.76</v>
       </c>
       <c r="I52" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J52" t="s" s="1">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="K52" t="n" s="185">
-        <v>4782859.0</v>
+        <v>4520320.5</v>
       </c>
     </row>
     <row r="53">
@@ -3669,25 +3669,25 @@
         <v>22</v>
       </c>
       <c r="E53" t="n" s="186">
-        <v>14434.0</v>
+        <v>13203.0</v>
       </c>
       <c r="F53" t="n" s="187">
-        <v>0.226609</v>
+        <v>0.211594</v>
       </c>
       <c r="G53" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H53" t="n" s="188">
-        <v>322.17</v>
+        <v>322.3</v>
       </c>
       <c r="I53" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J53" t="s" s="1">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="K53" t="n" s="189">
-        <v>4650202.0</v>
+        <v>4255327.0</v>
       </c>
     </row>
     <row r="54">
@@ -3704,25 +3704,25 @@
         <v>22</v>
       </c>
       <c r="E54" t="n" s="190">
-        <v>30949.0</v>
+        <v>17804.0</v>
       </c>
       <c r="F54" t="n" s="191">
-        <v>0.211054</v>
+        <v>0.192163</v>
       </c>
       <c r="G54" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H54" t="n" s="192">
-        <v>139.94</v>
+        <v>217.06</v>
       </c>
       <c r="I54" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J54" t="s" s="1">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="K54" t="n" s="193">
-        <v>4331003.0</v>
+        <v>3864536.3</v>
       </c>
     </row>
     <row r="55">
@@ -3739,25 +3739,25 @@
         <v>22</v>
       </c>
       <c r="E55" t="n" s="194">
-        <v>45559.0</v>
+        <v>30990.0</v>
       </c>
       <c r="F55" t="n" s="195">
-        <v>0.195949</v>
+        <v>0.186642</v>
       </c>
       <c r="G55" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H55" t="n" s="196">
-        <v>88.26</v>
+        <v>121.12</v>
       </c>
       <c r="I55" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J55" t="s" s="1">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="K55" t="n" s="197">
-        <v>4021037.3</v>
+        <v>3753508.8</v>
       </c>
     </row>
     <row r="56">
@@ -3774,25 +3774,25 @@
         <v>22</v>
       </c>
       <c r="E56" t="n" s="198">
-        <v>17780.0</v>
+        <v>45620.0</v>
       </c>
       <c r="F56" t="n" s="199">
-        <v>0.180721</v>
+        <v>0.185286</v>
       </c>
       <c r="G56" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H56" t="n" s="200">
-        <v>208.58</v>
+        <v>81.68</v>
       </c>
       <c r="I56" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J56" t="s" s="1">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K56" t="n" s="201">
-        <v>3708552.5</v>
+        <v>3726241.5</v>
       </c>
     </row>
     <row r="57">
@@ -3809,25 +3809,25 @@
         <v>22</v>
       </c>
       <c r="E57" t="n" s="202">
-        <v>32993.0</v>
+        <v>8502.0</v>
       </c>
       <c r="F57" t="n" s="203">
-        <v>0.157354</v>
+        <v>0.153973</v>
       </c>
       <c r="G57" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H57" t="n" s="204">
-        <v>97.87</v>
+        <v>364.21</v>
       </c>
       <c r="I57" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J57" t="s" s="1">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="K57" t="n" s="205">
-        <v>3229025.0</v>
+        <v>3096513.5</v>
       </c>
     </row>
     <row r="58">
@@ -3844,25 +3844,25 @@
         <v>22</v>
       </c>
       <c r="E58" t="n" s="206">
-        <v>8491.0</v>
+        <v>33037.0</v>
       </c>
       <c r="F58" t="n" s="207">
-        <v>0.147279</v>
+        <v>0.144759</v>
       </c>
       <c r="G58" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H58" t="n" s="208">
-        <v>355.94</v>
+        <v>88.12</v>
       </c>
       <c r="I58" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J58" t="s" s="1">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K58" t="n" s="209">
-        <v>3022286.5</v>
+        <v>2911220.5</v>
       </c>
     </row>
     <row r="59">
@@ -3879,25 +3879,25 @@
         <v>22</v>
       </c>
       <c r="E59" t="n" s="210">
-        <v>8884.0</v>
+        <v>8896.0</v>
       </c>
       <c r="F59" t="n" s="211">
-        <v>0.143952</v>
+        <v>0.135828</v>
       </c>
       <c r="G59" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H59" t="n" s="212">
-        <v>332.51</v>
+        <v>307.06</v>
       </c>
       <c r="I59" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J59" t="s" s="1">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="K59" t="n" s="213">
-        <v>2954018.8</v>
+        <v>2731605.8</v>
       </c>
     </row>
     <row r="60">
@@ -3914,16 +3914,16 @@
         <v>22</v>
       </c>
       <c r="E60" t="n" s="214">
-        <v>16610.0</v>
+        <v>16632.0</v>
       </c>
       <c r="F60" t="n" s="215">
-        <v>0.139002</v>
+        <v>0.132067</v>
       </c>
       <c r="G60" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H60" t="n" s="216">
-        <v>171.73</v>
+        <v>159.69</v>
       </c>
       <c r="I60" t="s" s="1">
         <v>24</v>
@@ -3932,7 +3932,7 @@
         <v>29</v>
       </c>
       <c r="K60" t="n" s="217">
-        <v>2852435.3</v>
+        <v>2655964.0</v>
       </c>
     </row>
     <row r="61">
@@ -3949,25 +3949,25 @@
         <v>22</v>
       </c>
       <c r="E61" t="n" s="218">
-        <v>17616.0</v>
+        <v>17174.0</v>
       </c>
       <c r="F61" t="n" s="219">
-        <v>0.123153</v>
+        <v>0.124193</v>
       </c>
       <c r="G61" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H61" t="n" s="220">
-        <v>143.46</v>
+        <v>145.43</v>
       </c>
       <c r="I61" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J61" t="s" s="1">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="K61" t="n" s="221">
-        <v>2527191.3</v>
+        <v>2497614.8</v>
       </c>
     </row>
     <row r="62">
@@ -3984,25 +3984,25 @@
         <v>22</v>
       </c>
       <c r="E62" t="n" s="222">
-        <v>1958.0</v>
+        <v>3902.0</v>
       </c>
       <c r="F62" t="n" s="223">
-        <v>0.122075</v>
+        <v>0.122403</v>
       </c>
       <c r="G62" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H62" t="n" s="224">
-        <v>1279.41</v>
+        <v>630.86</v>
       </c>
       <c r="I62" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J62" t="s" s="1">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="K62" t="n" s="225">
-        <v>2505084.8</v>
+        <v>2461615.8</v>
       </c>
     </row>
     <row r="63">
@@ -4019,25 +4019,25 @@
         <v>22</v>
       </c>
       <c r="E63" t="n" s="226">
-        <v>3897.0</v>
+        <v>1961.0</v>
       </c>
       <c r="F63" t="n" s="227">
-        <v>0.119929</v>
+        <v>0.121031</v>
       </c>
       <c r="G63" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H63" t="n" s="228">
-        <v>631.52</v>
+        <v>1241.22</v>
       </c>
       <c r="I63" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J63" t="s" s="1">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="K63" t="n" s="229">
-        <v>2461033.5</v>
+        <v>2434032.5</v>
       </c>
     </row>
     <row r="64">
@@ -4054,25 +4054,25 @@
         <v>22</v>
       </c>
       <c r="E64" t="n" s="230">
-        <v>17151.0</v>
+        <v>17639.0</v>
       </c>
       <c r="F64" t="n" s="231">
-        <v>0.115623</v>
+        <v>0.11882</v>
       </c>
       <c r="G64" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H64" t="n" s="232">
-        <v>138.34</v>
+        <v>135.47</v>
       </c>
       <c r="I64" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J64" t="s" s="1">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K64" t="n" s="233">
-        <v>2372669.3</v>
+        <v>2389555.3</v>
       </c>
     </row>
     <row r="65">
@@ -4089,16 +4089,16 @@
         <v>22</v>
       </c>
       <c r="E65" t="n" s="234">
-        <v>9045.0</v>
+        <v>9057.0</v>
       </c>
       <c r="F65" t="n" s="235">
-        <v>0.100716</v>
+        <v>0.095444</v>
       </c>
       <c r="G65" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H65" t="n" s="236">
-        <v>228.5</v>
+        <v>211.93</v>
       </c>
       <c r="I65" t="s" s="1">
         <v>24</v>
@@ -4107,7 +4107,7 @@
         <v>25</v>
       </c>
       <c r="K65" t="n" s="237">
-        <v>2066782.5</v>
+        <v>1919450.0</v>
       </c>
     </row>
     <row r="66">
@@ -4124,25 +4124,25 @@
         <v>22</v>
       </c>
       <c r="E66" t="n" s="238">
-        <v>4745.0</v>
+        <v>4751.0</v>
       </c>
       <c r="F66" t="n" s="239">
-        <v>0.099502</v>
+        <v>0.095302</v>
       </c>
       <c r="G66" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H66" t="n" s="240">
-        <v>430.32</v>
+        <v>403.41</v>
       </c>
       <c r="I66" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J66" t="s" s="1">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K66" t="n" s="241">
-        <v>2041868.4</v>
+        <v>1916600.9</v>
       </c>
     </row>
     <row r="67">
@@ -4159,25 +4159,25 @@
         <v>22</v>
       </c>
       <c r="E67" t="n" s="242">
-        <v>6892.0</v>
+        <v>6901.0</v>
       </c>
       <c r="F67" t="n" s="243">
-        <v>0.090674</v>
+        <v>0.094442</v>
       </c>
       <c r="G67" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H67" t="n" s="244">
-        <v>269.98</v>
+        <v>275.22</v>
       </c>
       <c r="I67" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J67" t="s" s="1">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="K67" t="n" s="245">
-        <v>1860702.1</v>
+        <v>1899293.3</v>
       </c>
     </row>
     <row r="68">
@@ -4194,16 +4194,16 @@
         <v>22</v>
       </c>
       <c r="E68" t="n" s="246">
-        <v>76997.0</v>
+        <v>77100.0</v>
       </c>
       <c r="F68" t="n" s="247">
-        <v>0.090539</v>
+        <v>0.092547</v>
       </c>
       <c r="G68" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H68" t="n" s="248">
-        <v>24.13</v>
+        <v>24.14</v>
       </c>
       <c r="I68" t="s" s="1">
         <v>24</v>
@@ -4212,7 +4212,7 @@
         <v>29</v>
       </c>
       <c r="K68" t="n" s="249">
-        <v>1857937.6</v>
+        <v>1861194.0</v>
       </c>
     </row>
     <row r="69">
@@ -4229,25 +4229,25 @@
         <v>22</v>
       </c>
       <c r="E69" t="n" s="250">
-        <v>39890.0</v>
+        <v>39943.0</v>
       </c>
       <c r="F69" t="n" s="251">
-        <v>0.084364</v>
+        <v>0.088503</v>
       </c>
       <c r="G69" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H69" t="n" s="252">
-        <v>43.4</v>
+        <v>44.56</v>
       </c>
       <c r="I69" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J69" t="s" s="1">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="K69" t="n" s="253">
-        <v>1731226.0</v>
+        <v>1779860.1</v>
       </c>
     </row>
     <row r="70">
@@ -4264,25 +4264,25 @@
         <v>22</v>
       </c>
       <c r="E70" t="n" s="254">
-        <v>12235.0</v>
+        <v>12251.0</v>
       </c>
       <c r="F70" t="n" s="255">
-        <v>0.077223</v>
+        <v>0.072376</v>
       </c>
       <c r="G70" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H70" t="n" s="256">
-        <v>129.52</v>
+        <v>118.81</v>
       </c>
       <c r="I70" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J70" t="s" s="1">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="K70" t="n" s="257">
-        <v>1584677.3</v>
+        <v>1455541.3</v>
       </c>
     </row>
     <row r="71">
@@ -4299,25 +4299,25 @@
         <v>22</v>
       </c>
       <c r="E71" t="n" s="258">
-        <v>10750.0</v>
+        <v>10764.0</v>
       </c>
       <c r="F71" t="n" s="259">
-        <v>0.07345</v>
+        <v>0.071904</v>
       </c>
       <c r="G71" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H71" t="n" s="260">
-        <v>140.21</v>
+        <v>134.34</v>
       </c>
       <c r="I71" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J71" t="s" s="1">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="K71" t="n" s="261">
-        <v>1507257.5</v>
+        <v>1446035.8</v>
       </c>
     </row>
     <row r="72">
@@ -4334,25 +4334,25 @@
         <v>22</v>
       </c>
       <c r="E72" t="n" s="262">
-        <v>47373.0</v>
+        <v>46463.0</v>
       </c>
       <c r="F72" t="n" s="263">
-        <v>0.065193</v>
+        <v>0.062403</v>
       </c>
       <c r="G72" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H72" t="n" s="264">
-        <v>28.24</v>
+        <v>27.01</v>
       </c>
       <c r="I72" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J72" t="s" s="1">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K72" t="n" s="265">
-        <v>1337813.5</v>
+        <v>1254965.6</v>
       </c>
     </row>
     <row r="73">
@@ -4369,16 +4369,16 @@
         <v>22</v>
       </c>
       <c r="E73" t="n" s="266">
-        <v>46401.0</v>
+        <v>9737.0</v>
       </c>
       <c r="F73" t="n" s="267">
-        <v>0.058768</v>
+        <v>0.061664</v>
       </c>
       <c r="G73" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H73" t="n" s="268">
-        <v>25.99</v>
+        <v>127.36</v>
       </c>
       <c r="I73" t="s" s="1">
         <v>24</v>
@@ -4387,7 +4387,7 @@
         <v>33</v>
       </c>
       <c r="K73" t="n" s="269">
-        <v>1205962.0</v>
+        <v>1240104.4</v>
       </c>
     </row>
     <row r="74">
@@ -4404,25 +4404,25 @@
         <v>22</v>
       </c>
       <c r="E74" t="n" s="270">
-        <v>9724.0</v>
+        <v>47436.0</v>
       </c>
       <c r="F74" t="n" s="271">
-        <v>0.058659</v>
+        <v>0.058214</v>
       </c>
       <c r="G74" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H74" t="n" s="272">
-        <v>123.79</v>
+        <v>24.68</v>
       </c>
       <c r="I74" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J74" t="s" s="1">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="K74" t="n" s="273">
-        <v>1203734.0</v>
+        <v>1170720.5</v>
       </c>
     </row>
     <row r="75">
@@ -4439,16 +4439,16 @@
         <v>22</v>
       </c>
       <c r="E75" t="n" s="274">
-        <v>3554.0</v>
+        <v>3559.0</v>
       </c>
       <c r="F75" t="n" s="275">
-        <v>0.053864</v>
+        <v>0.055963</v>
       </c>
       <c r="G75" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H75" t="n" s="276">
-        <v>311.01</v>
+        <v>316.23</v>
       </c>
       <c r="I75" t="s" s="1">
         <v>24</v>
@@ -4457,7 +4457,7 @@
         <v>33</v>
       </c>
       <c r="K75" t="n" s="277">
-        <v>1105329.5</v>
+        <v>1125462.6</v>
       </c>
     </row>
     <row r="76">
@@ -4474,25 +4474,25 @@
         <v>22</v>
       </c>
       <c r="E76" t="n" s="278">
-        <v>4005.0</v>
+        <v>11164.0</v>
       </c>
       <c r="F76" t="n" s="279">
-        <v>0.053212</v>
+        <v>0.053409</v>
       </c>
       <c r="G76" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H76" t="n" s="280">
-        <v>272.65</v>
+        <v>96.21</v>
       </c>
       <c r="I76" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J76" t="s" s="1">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K76" t="n" s="281">
-        <v>1091963.3</v>
+        <v>1074088.5</v>
       </c>
     </row>
     <row r="77">
@@ -4509,25 +4509,25 @@
         <v>22</v>
       </c>
       <c r="E77" t="n" s="282">
-        <v>19622.0</v>
+        <v>4010.0</v>
       </c>
       <c r="F77" t="n" s="283">
-        <v>0.050401</v>
+        <v>0.052848</v>
       </c>
       <c r="G77" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H77" t="n" s="284">
-        <v>52.71</v>
+        <v>265.04</v>
       </c>
       <c r="I77" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J77" t="s" s="1">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="K77" t="n" s="285">
-        <v>1034275.6</v>
+        <v>1062810.4</v>
       </c>
     </row>
     <row r="78">
@@ -4544,25 +4544,25 @@
         <v>22</v>
       </c>
       <c r="E78" t="n" s="286">
-        <v>11149.0</v>
+        <v>19648.0</v>
       </c>
       <c r="F78" t="n" s="287">
-        <v>0.04774</v>
+        <v>0.052513</v>
       </c>
       <c r="G78" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H78" t="n" s="288">
-        <v>87.87</v>
+        <v>53.75</v>
       </c>
       <c r="I78" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J78" t="s" s="1">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="K78" t="n" s="289">
-        <v>979662.6</v>
+        <v>1056080.0</v>
       </c>
     </row>
     <row r="79">
@@ -4579,25 +4579,25 @@
         <v>22</v>
       </c>
       <c r="E79" t="n" s="290">
-        <v>12664.0</v>
+        <v>5651.0</v>
       </c>
       <c r="F79" t="n" s="291">
-        <v>0.036997</v>
+        <v>0.040151</v>
       </c>
       <c r="G79" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H79" t="n" s="292">
-        <v>59.95</v>
+        <v>142.89</v>
       </c>
       <c r="I79" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J79" t="s" s="1">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="K79" t="n" s="293">
-        <v>759206.8</v>
+        <v>807471.4</v>
       </c>
     </row>
     <row r="80">
@@ -4614,25 +4614,25 @@
         <v>22</v>
       </c>
       <c r="E80" t="n" s="294">
-        <v>5643.0</v>
+        <v>12681.0</v>
       </c>
       <c r="F80" t="n" s="295">
-        <v>0.036488</v>
+        <v>0.036339</v>
       </c>
       <c r="G80" t="s" s="1">
         <v>23</v>
       </c>
       <c r="H80" t="n" s="296">
-        <v>132.69</v>
+        <v>57.63</v>
       </c>
       <c r="I80" t="s" s="1">
         <v>24</v>
       </c>
       <c r="J80" t="s" s="1">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="K80" t="n" s="297">
-        <v>748769.7</v>
+        <v>730806.0</v>
       </c>
     </row>
     <row r="81">
@@ -4658,7 +4658,7 @@
         <v>253</v>
       </c>
       <c r="H81" t="n" s="299">
-        <v>376080.0</v>
+        <v>360090.0</v>
       </c>
       <c r="I81" t="s" s="1">
         <v>250</v>
@@ -4667,7 +4667,7 @@
         <v>250</v>
       </c>
       <c r="K81" t="n" s="300">
-        <v>752160.0</v>
+        <v>720180.0</v>
       </c>
     </row>
     <row r="82">
@@ -4702,7 +4702,7 @@
         <v>250</v>
       </c>
       <c r="K82" t="n" s="303">
-        <v>2016.2014</v>
+        <v>2018.0531</v>
       </c>
     </row>
     <row r="83">
@@ -4719,7 +4719,7 @@
         <v>22</v>
       </c>
       <c r="E83" t="n" s="304">
-        <v>1627192.0</v>
+        <v>1650766.0</v>
       </c>
       <c r="F83" t="s" s="1">
         <v>252</v>
@@ -4737,7 +4737,7 @@
         <v>250</v>
       </c>
       <c r="K83" t="n" s="306">
-        <v>1627191.9</v>
+        <v>1650765.9</v>
       </c>
     </row>
     <row r="84"/>

</xml_diff>